<commit_message>
Updated KEN_grids_kan model - 2025-11-30 00:22
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD6D86CD-5520-4E35-8742-BBE3685709CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A818AFB1-8A4C-4B72-BD72-9010DB88CD8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1757,7 +1757,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C6A49291-04FA-4433-8C17-F12DC5606A33}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D9D9A34-9132-41DB-9483-8FDEC94553F2}">
   <dimension ref="B9:E105"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-06 18:05
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{061DFF0B-5E86-45BA-9149-197B97D553A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFCEC161-77DB-4763-BFC0-B57F239197BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1757,7 +1757,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42880EB5-1E1C-4F11-B662-560472C1CB1C}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD6874D9-5B1C-4EA0-A9FD-D2EA98E90CCA}">
   <dimension ref="B9:E105"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2025-12-11 11:15
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DFCEC161-77DB-4763-BFC0-B57F239197BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3274AEF6-5F7D-40D7-8C28-68CA2D371B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1757,7 +1757,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD6874D9-5B1C-4EA0-A9FD-D2EA98E90CCA}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{454C2055-16E0-401F-83D7-57F5EAAC86DF}">
   <dimension ref="B9:E105"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>

</xml_diff>

<commit_message>
Updated KEN_grids_kan model - 2026-06-25 19:22
</commit_message>
<xml_diff>
--- a/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
+++ b/VerveStacks_KEN_grids_kan/Sets-vervestacks.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr updateLinks="never" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_KEN_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{17E5577D-9B8A-44CA-A880-5AEDB1F6554A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{63B5AE75-D709-45F0-A330-21BBC5E67A6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="309">
   <si>
     <t>~TFM_Psets</t>
   </si>
@@ -313,25 +313,40 @@
     <t>distr*</t>
   </si>
   <si>
-    <t>e*[_]gas_combined_cycle*,e*[_]oil_combined_cycle*,CCGT*,*GasCC*</t>
-  </si>
-  <si>
     <t>e*[_]gas_internal_combustion*,e*[_]oil_internal_combustion*</t>
   </si>
   <si>
     <t>e*[_]gas_steam_turbine*,e*[_]oil_steam_turbine*</t>
   </si>
   <si>
-    <t>e*[_]gas_gas_turbine*,e*[_]oil_gas_turbine*,gas turbine*,EN*CT*</t>
-  </si>
-  <si>
     <t>e*[_]coal_CFB*,e*[_]coal_subcritical*,*subcritical*</t>
   </si>
   <si>
+    <t>ELE,CHP</t>
+  </si>
+  <si>
+    <t>bio*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_combined_cycle*,e*[_]oil_combined_cycle*,*CCGT*,*GasCC*</t>
+  </si>
+  <si>
+    <t>e*[_]gas_gas_turbine*,e*[_]oil_gas_turbine*,*gas*turbine*,EN*CT*</t>
+  </si>
+  <si>
     <t>e*[_]coal_supercritical*,e*[_]coal_supercritical_CCS*,e*[_]coal_ultra-supercritical*,e*[_]coal_ultra-supercritical_CCS*,*supercritical*</t>
   </si>
   <si>
-    <t>e*[_]bioenergy*,bioen*</t>
+    <t>distr_sol*</t>
+  </si>
+  <si>
+    <t>distr_won*</t>
+  </si>
+  <si>
+    <t>distr_wof*</t>
+  </si>
+  <si>
+    <t>coal</t>
   </si>
   <si>
     <t>~tfm_psets</t>
@@ -349,577 +364,607 @@
     <t>t_pos_andor</t>
   </si>
   <si>
-    <t>p_w86402221</t>
-  </si>
-  <si>
-    <t>e_w86402221*</t>
+    <t>p_w86402221-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w86402221-220_KEN*</t>
   </si>
   <si>
     <t>OR</t>
   </si>
   <si>
-    <t>p_w180021151</t>
-  </si>
-  <si>
-    <t>e_w180021151*</t>
-  </si>
-  <si>
-    <t>p_w220540545</t>
-  </si>
-  <si>
-    <t>e_w220540545*</t>
-  </si>
-  <si>
-    <t>p_w579310367</t>
-  </si>
-  <si>
-    <t>e_w579310367*</t>
-  </si>
-  <si>
-    <t>p_w457973270</t>
-  </si>
-  <si>
-    <t>e_w457973270*</t>
-  </si>
-  <si>
-    <t>p_w563813243</t>
-  </si>
-  <si>
-    <t>e_w563813243*</t>
-  </si>
-  <si>
-    <t>p_w569997185</t>
-  </si>
-  <si>
-    <t>e_w569997185*</t>
-  </si>
-  <si>
-    <t>p_w578140339</t>
-  </si>
-  <si>
-    <t>e_w578140339*</t>
-  </si>
-  <si>
-    <t>p_w659874569</t>
-  </si>
-  <si>
-    <t>e_w659874569*</t>
-  </si>
-  <si>
-    <t>p_w660091166</t>
-  </si>
-  <si>
-    <t>e_w660091166*</t>
-  </si>
-  <si>
-    <t>p_w665372427</t>
-  </si>
-  <si>
-    <t>e_w665372427*</t>
-  </si>
-  <si>
-    <t>p_w846713577</t>
-  </si>
-  <si>
-    <t>e_w846713577*</t>
-  </si>
-  <si>
-    <t>p_w669510376</t>
-  </si>
-  <si>
-    <t>e_w669510376*</t>
-  </si>
-  <si>
-    <t>p_w669520367</t>
-  </si>
-  <si>
-    <t>e_w669520367*</t>
-  </si>
-  <si>
-    <t>p_w696445754</t>
-  </si>
-  <si>
-    <t>e_w696445754*</t>
-  </si>
-  <si>
-    <t>p_w870818913</t>
-  </si>
-  <si>
-    <t>e_w870818913*</t>
-  </si>
-  <si>
-    <t>p_w953567827</t>
-  </si>
-  <si>
-    <t>e_w953567827*</t>
-  </si>
-  <si>
-    <t>p_w1115312336</t>
-  </si>
-  <si>
-    <t>e_w1115312336*</t>
-  </si>
-  <si>
-    <t>p_r14923640</t>
-  </si>
-  <si>
-    <t>e_r14923640*</t>
-  </si>
-  <si>
-    <t>p_KE7</t>
-  </si>
-  <si>
-    <t>e_KE7*</t>
-  </si>
-  <si>
-    <t>p_KE13</t>
-  </si>
-  <si>
-    <t>e_KE13*</t>
-  </si>
-  <si>
-    <t>p_KE2</t>
-  </si>
-  <si>
-    <t>e_KE2*</t>
-  </si>
-  <si>
-    <t>p_KE1</t>
-  </si>
-  <si>
-    <t>e_KE1*</t>
-  </si>
-  <si>
-    <t>p_KE8</t>
-  </si>
-  <si>
-    <t>e_KE8*</t>
-  </si>
-  <si>
-    <t>p_KE9</t>
-  </si>
-  <si>
-    <t>e_KE9*</t>
-  </si>
-  <si>
-    <t>p_KE14</t>
-  </si>
-  <si>
-    <t>e_KE14*</t>
-  </si>
-  <si>
-    <t>p_KE4</t>
-  </si>
-  <si>
-    <t>e_KE4*</t>
-  </si>
-  <si>
-    <t>p_KE10</t>
-  </si>
-  <si>
-    <t>e_KE10*</t>
-  </si>
-  <si>
-    <t>p_KE15</t>
-  </si>
-  <si>
-    <t>e_KE15*</t>
-  </si>
-  <si>
-    <t>p_KE6</t>
-  </si>
-  <si>
-    <t>e_KE6*</t>
-  </si>
-  <si>
-    <t>p_KE11</t>
-  </si>
-  <si>
-    <t>e_KE11*</t>
-  </si>
-  <si>
-    <t>p_KE3</t>
-  </si>
-  <si>
-    <t>e_KE3*</t>
-  </si>
-  <si>
-    <t>p_KE5</t>
-  </si>
-  <si>
-    <t>e_KE5*</t>
-  </si>
-  <si>
-    <t>p_KE12</t>
-  </si>
-  <si>
-    <t>e_KE12*</t>
-  </si>
-  <si>
-    <t>rez_spv_001</t>
-  </si>
-  <si>
-    <t>elc_spv_001</t>
-  </si>
-  <si>
-    <t>rez_spv_002</t>
-  </si>
-  <si>
-    <t>elc_spv_002</t>
-  </si>
-  <si>
-    <t>rez_spv_003</t>
-  </si>
-  <si>
-    <t>elc_spv_003</t>
-  </si>
-  <si>
-    <t>rez_spv_004</t>
-  </si>
-  <si>
-    <t>elc_spv_004</t>
-  </si>
-  <si>
-    <t>rez_spv_005</t>
-  </si>
-  <si>
-    <t>elc_spv_005</t>
-  </si>
-  <si>
-    <t>rez_spv_006</t>
-  </si>
-  <si>
-    <t>elc_spv_006</t>
-  </si>
-  <si>
-    <t>rez_spv_007</t>
-  </si>
-  <si>
-    <t>elc_spv_007</t>
-  </si>
-  <si>
-    <t>rez_spv_008</t>
-  </si>
-  <si>
-    <t>elc_spv_008</t>
-  </si>
-  <si>
-    <t>rez_spv_009</t>
-  </si>
-  <si>
-    <t>elc_spv_009</t>
-  </si>
-  <si>
-    <t>rez_spv_010</t>
-  </si>
-  <si>
-    <t>elc_spv_010</t>
-  </si>
-  <si>
-    <t>rez_spv_011</t>
-  </si>
-  <si>
-    <t>elc_spv_011</t>
-  </si>
-  <si>
-    <t>rez_spv_012</t>
-  </si>
-  <si>
-    <t>elc_spv_012</t>
-  </si>
-  <si>
-    <t>rez_spv_013</t>
-  </si>
-  <si>
-    <t>elc_spv_013</t>
-  </si>
-  <si>
-    <t>rez_spv_014</t>
-  </si>
-  <si>
-    <t>elc_spv_014</t>
-  </si>
-  <si>
-    <t>rez_spv_015</t>
-  </si>
-  <si>
-    <t>elc_spv_015</t>
-  </si>
-  <si>
-    <t>rez_spv_016</t>
-  </si>
-  <si>
-    <t>elc_spv_016</t>
-  </si>
-  <si>
-    <t>rez_spv_017</t>
-  </si>
-  <si>
-    <t>elc_spv_017</t>
-  </si>
-  <si>
-    <t>rez_spv_018</t>
-  </si>
-  <si>
-    <t>elc_spv_018</t>
-  </si>
-  <si>
-    <t>rez_spv_019</t>
-  </si>
-  <si>
-    <t>elc_spv_019</t>
-  </si>
-  <si>
-    <t>rez_spv_020</t>
-  </si>
-  <si>
-    <t>elc_spv_020</t>
-  </si>
-  <si>
-    <t>rez_spv_021</t>
-  </si>
-  <si>
-    <t>elc_spv_021</t>
-  </si>
-  <si>
-    <t>rez_spv_022</t>
-  </si>
-  <si>
-    <t>elc_spv_022</t>
-  </si>
-  <si>
-    <t>rez_spv_023</t>
-  </si>
-  <si>
-    <t>elc_spv_023</t>
-  </si>
-  <si>
-    <t>rez_spv_024</t>
-  </si>
-  <si>
-    <t>elc_spv_024</t>
-  </si>
-  <si>
-    <t>rez_spv_025</t>
-  </si>
-  <si>
-    <t>elc_spv_025</t>
-  </si>
-  <si>
-    <t>rez_spv_026</t>
-  </si>
-  <si>
-    <t>elc_spv_026</t>
-  </si>
-  <si>
-    <t>rez_spv_027</t>
-  </si>
-  <si>
-    <t>elc_spv_027</t>
-  </si>
-  <si>
-    <t>rez_spv_028</t>
-  </si>
-  <si>
-    <t>elc_spv_028</t>
-  </si>
-  <si>
-    <t>rez_won_001</t>
-  </si>
-  <si>
-    <t>elc_won_001</t>
-  </si>
-  <si>
-    <t>rez_won_002</t>
-  </si>
-  <si>
-    <t>elc_won_002</t>
-  </si>
-  <si>
-    <t>rez_won_003</t>
-  </si>
-  <si>
-    <t>elc_won_003</t>
-  </si>
-  <si>
-    <t>rez_won_004</t>
-  </si>
-  <si>
-    <t>elc_won_004</t>
-  </si>
-  <si>
-    <t>rez_won_005</t>
-  </si>
-  <si>
-    <t>elc_won_005</t>
-  </si>
-  <si>
-    <t>rez_won_006</t>
-  </si>
-  <si>
-    <t>elc_won_006</t>
-  </si>
-  <si>
-    <t>rez_won_007</t>
-  </si>
-  <si>
-    <t>elc_won_007</t>
-  </si>
-  <si>
-    <t>rez_won_008</t>
-  </si>
-  <si>
-    <t>elc_won_008</t>
-  </si>
-  <si>
-    <t>rez_won_009</t>
-  </si>
-  <si>
-    <t>elc_won_009</t>
-  </si>
-  <si>
-    <t>rez_won_010</t>
-  </si>
-  <si>
-    <t>elc_won_010</t>
-  </si>
-  <si>
-    <t>rez_won_011</t>
-  </si>
-  <si>
-    <t>elc_won_011</t>
-  </si>
-  <si>
-    <t>rez_won_012</t>
-  </si>
-  <si>
-    <t>elc_won_012</t>
-  </si>
-  <si>
-    <t>rez_won_013</t>
-  </si>
-  <si>
-    <t>elc_won_013</t>
-  </si>
-  <si>
-    <t>rez_won_014</t>
-  </si>
-  <si>
-    <t>elc_won_014</t>
-  </si>
-  <si>
-    <t>rez_won_015</t>
-  </si>
-  <si>
-    <t>elc_won_015</t>
-  </si>
-  <si>
-    <t>rez_won_016</t>
-  </si>
-  <si>
-    <t>elc_won_016</t>
-  </si>
-  <si>
-    <t>rez_won_017</t>
-  </si>
-  <si>
-    <t>elc_won_017</t>
-  </si>
-  <si>
-    <t>rez_won_018</t>
-  </si>
-  <si>
-    <t>elc_won_018</t>
-  </si>
-  <si>
-    <t>rez_won_019</t>
-  </si>
-  <si>
-    <t>elc_won_019</t>
-  </si>
-  <si>
-    <t>rez_won_020</t>
-  </si>
-  <si>
-    <t>elc_won_020</t>
-  </si>
-  <si>
-    <t>rez_won_021</t>
-  </si>
-  <si>
-    <t>elc_won_021</t>
-  </si>
-  <si>
-    <t>rez_won_022</t>
-  </si>
-  <si>
-    <t>elc_won_022</t>
-  </si>
-  <si>
-    <t>rez_won_023</t>
-  </si>
-  <si>
-    <t>elc_won_023</t>
-  </si>
-  <si>
-    <t>rez_wof_001</t>
-  </si>
-  <si>
-    <t>elc_wof_001</t>
-  </si>
-  <si>
-    <t>rez_wof_002</t>
-  </si>
-  <si>
-    <t>elc_wof_002</t>
-  </si>
-  <si>
-    <t>rez_wof_003</t>
-  </si>
-  <si>
-    <t>elc_wof_003</t>
-  </si>
-  <si>
-    <t>rez_wof_004</t>
-  </si>
-  <si>
-    <t>elc_wof_004</t>
-  </si>
-  <si>
-    <t>rez_wof_005</t>
-  </si>
-  <si>
-    <t>elc_wof_005</t>
-  </si>
-  <si>
-    <t>rez_wof_006</t>
-  </si>
-  <si>
-    <t>elc_wof_006</t>
-  </si>
-  <si>
-    <t>rez_wof_007</t>
-  </si>
-  <si>
-    <t>elc_wof_007</t>
-  </si>
-  <si>
-    <t>rez_wof_008</t>
-  </si>
-  <si>
-    <t>elc_wof_008</t>
-  </si>
-  <si>
-    <t>rez_wof_009</t>
-  </si>
-  <si>
-    <t>elc_wof_009</t>
-  </si>
-  <si>
-    <t>rez_wof_010</t>
-  </si>
-  <si>
-    <t>elc_wof_010</t>
+    <t>p_w180021151-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w180021151-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w220540545-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w220540545-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w579310367-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w579310367-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w457973270-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w457973270-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w563813243-400_KEN</t>
+  </si>
+  <si>
+    <t>e_w563813243-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_w569997185-400_KEN</t>
+  </si>
+  <si>
+    <t>e_w569997185-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_w569997185-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w569997185-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w578140339-400_KEN</t>
+  </si>
+  <si>
+    <t>e_w578140339-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_w578140339-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w578140339-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w659874569-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w659874569-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w660091166-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w660091166-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w665372427-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w665372427-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w846713577-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w846713577-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w669510376-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w669510376-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w669520367-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w669520367-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w696445754-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w696445754-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w870818913-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w870818913-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w953567827-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w953567827-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w1115312336-220_KEN</t>
+  </si>
+  <si>
+    <t>e_w1115312336-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w870818913-400_KEN</t>
+  </si>
+  <si>
+    <t>e_w870818913-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_r14923640-220_KEN</t>
+  </si>
+  <si>
+    <t>e_r14923640-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE7-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE7-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE13-400_KEN</t>
+  </si>
+  <si>
+    <t>e_KE13-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE2-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE2-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE1-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE1-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE8-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE8-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE9-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE9-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_r14923640-400_KEN</t>
+  </si>
+  <si>
+    <t>e_r14923640-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE14-400_KEN</t>
+  </si>
+  <si>
+    <t>e_KE14-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE4-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE4-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE10-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE10-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE15-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE15-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE6-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE6-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE11-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE11-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE3-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE3-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_w457973270-400_KEN</t>
+  </si>
+  <si>
+    <t>e_w457973270-400_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE5-220_KEN</t>
+  </si>
+  <si>
+    <t>e_KE5-220_KEN*</t>
+  </si>
+  <si>
+    <t>p_KE12-400_KEN</t>
+  </si>
+  <si>
+    <t>e_KE12-400_KEN*</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_001</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_001</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_002</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_002</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_003</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_003</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_004</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_004</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_005</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_005</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_006</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_006</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_007</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_007</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_008</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_008</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_009</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_009</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_010</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_010</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_011</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_011</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_012</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_012</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_013</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_013</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_014</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_014</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_015</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_015</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_016</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_016</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_017</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_017</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_018</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_018</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_019</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_019</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_020</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_020</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_021</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_021</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_022</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_022</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_023</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_023</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_024</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_024</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_025</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_025</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_026</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_026</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_027</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_027</t>
+  </si>
+  <si>
+    <t>rez_spv_KEN_028</t>
+  </si>
+  <si>
+    <t>elc_spv_KEN_028</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_001</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_001</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_002</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_002</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_003</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_003</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_004</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_004</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_005</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_005</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_006</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_006</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_007</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_007</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_008</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_008</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_009</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_009</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_010</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_010</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_011</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_011</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_012</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_012</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_013</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_013</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_014</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_014</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_015</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_015</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_016</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_016</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_017</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_017</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_018</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_018</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_019</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_019</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_020</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_020</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_021</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_021</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_022</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_022</t>
+  </si>
+  <si>
+    <t>rez_won_KEN_023</t>
+  </si>
+  <si>
+    <t>elc_won_KEN_023</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_001</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_001</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_002</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_002</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_003</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_003</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_004</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_004</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_005</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_005</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_006</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_006</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_007</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_007</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_008</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_008</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_009</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_009</t>
+  </si>
+  <si>
+    <t>rez_wof_KEN_010</t>
+  </si>
+  <si>
+    <t>elc_wof_KEN_010</t>
   </si>
 </sst>
 </file>
@@ -951,12 +996,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -991,11 +1042,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="2"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Heading 2" xfId="1" builtinId="17"/>
@@ -1757,1357 +1809,1427 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3063124-3A9A-441F-8A51-0BA1B3ADA49E}">
-  <dimension ref="B9:E105"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D682EDA7-F1C5-439D-87DE-24679B76C4E0}">
+  <dimension ref="B9:E110"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <sheetData>
     <row r="9" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B10" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D10" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="E10" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E11" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B12" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C12" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D12" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="E12" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B13" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C13" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D13" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B14" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="D14" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="E14" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B15" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D15" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="E15" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B16" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D16" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="E16" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B17" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="C17" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D17" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="E17" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B18" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="C18" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D18" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="E18" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B19" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="C19" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D19" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E19" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B20" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="C20" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D20" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E20" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B21" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="C21" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D21" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E21" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B22" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="C22" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D22" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="E22" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B23" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="C23" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D23" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="E23" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B24" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C24" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D24" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="E24" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B25" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="C25" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="D25" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="E25" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B26" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C26" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D26" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="E26" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="27" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B27" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="C27" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="D27" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="E27" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B28" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C28" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D28" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="E28" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B29" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C29" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D29" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="E29" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B30" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C30" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D30" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="E30" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B31" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C31" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D31" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E31" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B32" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C32" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D32" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="E32" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="33" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B33" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C33" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D33" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E33" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="34" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B34" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C34" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D34" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="E34" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="35" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B35" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C35" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D35" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E35" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="36" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B36" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C36" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D36" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="E36" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="37" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B37" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C37" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D37" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E37" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B38" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C38" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D38" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="E38" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="39" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B39" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="C39" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="D39" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E39" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="40" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B40" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="C40" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="D40" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="E40" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B41" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C41" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D41" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="E41" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="42" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B42" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C42" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D42" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="E42" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="43" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B43" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C43" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D43" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="E43" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="44" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B44" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C44" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D44" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="E44" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="45" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B45" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C45" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D45" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="E45" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="46" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B46" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C46" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D46" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="E46" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="47" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B47" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C47" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="D47" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="E47" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B48" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C48" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="D48" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="E48" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B49" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C49" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D49" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="E49" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B50" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="C50" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="D50" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="E50" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B51" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="C51" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="D51" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E51" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B52" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="C52" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="D52" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="E52" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B53" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C53" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="D53" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="E53" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B54" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C54" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="D54" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E54" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B55" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C55" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D55" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="E55" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B56" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C56" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="D56" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="E56" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B57" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C57" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D57" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="E57" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B58" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="C58" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="D58" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="E58" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B59" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="C59" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="D59" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="E59" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B60" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="C60" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D60" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E60" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B61" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C61" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="D61" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E61" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="62" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B62" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="C62" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="D62" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="E62" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="63" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B63" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C63" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D63" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="E63" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="64" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B64" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="C64" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="D64" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="E64" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="65" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B65" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C65" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D65" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="E65" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="66" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B66" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C66" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D66" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="E66" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="67" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B67" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="C67" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="D67" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="E67" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B68" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C68" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="D68" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="E68" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B69" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C69" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="D69" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E69" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B70" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="C70" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="D70" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="E70" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B71" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="C71" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="D71" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="E71" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B72" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="C72" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="D72" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="E72" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B73" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C73" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D73" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="E73" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B74" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="C74" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="D74" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="E74" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B75" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C75" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="D75" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="E75" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B76" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="C76" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="D76" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="E76" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B77" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C77" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D77" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E77" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B78" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="C78" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="D78" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="E78" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B79" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C79" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D79" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="E79" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B80" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="C80" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="D80" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E80" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B81" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C81" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D81" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E81" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="82" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B82" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="C82" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="D82" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="E82" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="83" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B83" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="C83" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D83" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="E83" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="84" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B84" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="C84" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="D84" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="E84" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="85" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B85" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C85" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D85" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="E85" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="86" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B86" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C86" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="D86" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E86" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="87" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B87" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C87" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="D87" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E87" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="88" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B88" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C88" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D88" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E88" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="89" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B89" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C89" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="D89" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="E89" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="90" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B90" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C90" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D90" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="E90" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="91" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B91" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C91" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D91" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="E91" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B92" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C92" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D92" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="E92" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B93" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C93" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="D93" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E93" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B94" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C94" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="D94" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="E94" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B95" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C95" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D95" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="E95" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B96" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="C96" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="D96" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="E96" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B97" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C97" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="D97" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E97" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B98" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="C98" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="D98" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="E98" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B99" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="C99" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="D99" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="E99" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="100" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B100" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="C100" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="D100" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="E100" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B101" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="C101" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="D101" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E101" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="102" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B102" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C102" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="D102" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E102" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="103" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B103" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C103" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D103" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="E103" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="104" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B104" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="C104" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="D104" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="E104" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="105" spans="2:5" x14ac:dyDescent="0.45">
       <c r="B105" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C105" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="D105" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="E105" t="s">
-        <v>105</v>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="106" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B106" t="s">
+        <v>299</v>
+      </c>
+      <c r="C106" t="s">
+        <v>300</v>
+      </c>
+      <c r="D106" t="s">
+        <v>300</v>
+      </c>
+      <c r="E106" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="107" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B107" t="s">
+        <v>301</v>
+      </c>
+      <c r="C107" t="s">
+        <v>302</v>
+      </c>
+      <c r="D107" t="s">
+        <v>302</v>
+      </c>
+      <c r="E107" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="108" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B108" t="s">
+        <v>303</v>
+      </c>
+      <c r="C108" t="s">
+        <v>304</v>
+      </c>
+      <c r="D108" t="s">
+        <v>304</v>
+      </c>
+      <c r="E108" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B109" t="s">
+        <v>305</v>
+      </c>
+      <c r="C109" t="s">
+        <v>306</v>
+      </c>
+      <c r="D109" t="s">
+        <v>306</v>
+      </c>
+      <c r="E109" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="110" spans="2:5" x14ac:dyDescent="0.45">
+      <c r="B110" t="s">
+        <v>307</v>
+      </c>
+      <c r="C110" t="s">
+        <v>308</v>
+      </c>
+      <c r="D110" t="s">
+        <v>308</v>
+      </c>
+      <c r="E110" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>
@@ -3117,7 +3239,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71754C8A-E599-4286-919F-11B5789CC171}">
-  <dimension ref="A1:K48"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="86" bestFit="1" customWidth="1"/>
@@ -3166,7 +3288,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B3" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -3183,7 +3305,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="F4" t="s">
         <v>28</v>
@@ -3191,7 +3313,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F5" t="s">
         <v>27</v>
@@ -3199,7 +3321,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B6" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="F6" t="s">
         <v>19</v>
@@ -3213,7 +3335,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F7" t="s">
         <v>20</v>
@@ -3221,7 +3343,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="B8" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="F8" t="s">
         <v>21</v>
@@ -3236,8 +3358,11 @@
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.45">
-      <c r="B10" t="s">
-        <v>97</v>
+      <c r="A10" t="s">
+        <v>94</v>
+      </c>
+      <c r="D10" t="s">
+        <v>95</v>
       </c>
       <c r="F10" t="s">
         <v>68</v>
@@ -3419,292 +3544,109 @@
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B26" t="str">
-        <f>"g[_]*"&amp;K26</f>
-        <v>g[_]*220</v>
-      </c>
-      <c r="F26" t="str">
-        <f>"Grid-"&amp;K26&amp;"V"</f>
-        <v>Grid-220V</v>
+      <c r="B26" t="s">
+        <v>90</v>
+      </c>
+      <c r="F26" t="s">
+        <v>78</v>
       </c>
       <c r="K26">
         <v>220</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B27" t="str">
-        <f t="shared" ref="B27:B46" si="0">"g[_]*"&amp;K27</f>
-        <v>g[_]*400</v>
-      </c>
-      <c r="F27" t="str">
-        <f t="shared" ref="F27:F46" si="1">"Grid-"&amp;K27&amp;"V"</f>
-        <v>Grid-400V</v>
+      <c r="B27" t="s">
+        <v>79</v>
+      </c>
+      <c r="F27" t="s">
+        <v>80</v>
       </c>
       <c r="K27">
         <v>400</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B28" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*380</v>
-      </c>
-      <c r="F28" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-380V</v>
+      <c r="B28" t="s">
+        <v>99</v>
+      </c>
+      <c r="F28" s="4" t="str">
+        <f>LEFT(B28,9)</f>
+        <v>distr_sol</v>
       </c>
       <c r="K28">
         <v>380</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B29" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*225</v>
-      </c>
-      <c r="F29" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-225V</v>
+      <c r="B29" t="s">
+        <v>100</v>
+      </c>
+      <c r="F29" s="4" t="str">
+        <f t="shared" ref="F29:F30" si="0">LEFT(B29,9)</f>
+        <v>distr_won</v>
       </c>
       <c r="K29">
         <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B30" t="str">
+      <c r="B30" t="s">
+        <v>101</v>
+      </c>
+      <c r="F30" s="4" t="str">
         <f t="shared" si="0"/>
-        <v>g[_]*330</v>
-      </c>
-      <c r="F30" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-330V</v>
+        <v>distr_wof</v>
       </c>
       <c r="K30">
         <v>330</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B31" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*275</v>
-      </c>
-      <c r="F31" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-275V</v>
+      <c r="D31" t="s">
+        <v>34</v>
+      </c>
+      <c r="F31" s="4" t="str">
+        <f>"hs_"&amp;D31</f>
+        <v>hs_geothermal</v>
       </c>
       <c r="K31">
         <v>275</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.45">
-      <c r="B32" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*420</v>
-      </c>
-      <c r="F32" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-420V</v>
+      <c r="D32" t="s">
+        <v>35</v>
+      </c>
+      <c r="F32" s="4" t="str">
+        <f t="shared" ref="F32:F34" si="1">"hs_"&amp;D32</f>
+        <v>hs_hydro</v>
       </c>
       <c r="K32">
         <v>420</v>
       </c>
     </row>
-    <row r="33" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B33" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*300</v>
-      </c>
-      <c r="F33" t="str">
+    <row r="33" spans="4:11" x14ac:dyDescent="0.45">
+      <c r="D33" t="s">
+        <v>36</v>
+      </c>
+      <c r="F33" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Grid-300V</v>
+        <v>hs_nuclear</v>
       </c>
       <c r="K33">
         <v>300</v>
       </c>
     </row>
-    <row r="34" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B34" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*500</v>
-      </c>
-      <c r="F34" t="str">
+    <row r="34" spans="4:11" x14ac:dyDescent="0.45">
+      <c r="D34" t="s">
+        <v>102</v>
+      </c>
+      <c r="F34" s="4" t="str">
         <f t="shared" si="1"/>
-        <v>Grid-500V</v>
+        <v>hs_coal</v>
       </c>
       <c r="K34">
         <v>500</v>
-      </c>
-    </row>
-    <row r="35" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B35" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*750</v>
-      </c>
-      <c r="F35" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-750V</v>
-      </c>
-      <c r="K35">
-        <v>750</v>
-      </c>
-    </row>
-    <row r="36" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B36" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*450</v>
-      </c>
-      <c r="F36" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-450V</v>
-      </c>
-      <c r="K36">
-        <v>450</v>
-      </c>
-    </row>
-    <row r="37" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B37" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*515</v>
-      </c>
-      <c r="F37" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-515V</v>
-      </c>
-      <c r="K37">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="38" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B38" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*525</v>
-      </c>
-      <c r="F38" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-525V</v>
-      </c>
-      <c r="K38">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="39" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B39" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*320</v>
-      </c>
-      <c r="F39" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-320V</v>
-      </c>
-      <c r="K39">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="40" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B40" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*150</v>
-      </c>
-      <c r="F40" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-150V</v>
-      </c>
-      <c r="K40">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="41" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B41" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*270</v>
-      </c>
-      <c r="F41" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-270V</v>
-      </c>
-      <c r="K41">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="42" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B42" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*350</v>
-      </c>
-      <c r="F42" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-350V</v>
-      </c>
-      <c r="K42">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="43" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B43" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*250</v>
-      </c>
-      <c r="F43" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-250V</v>
-      </c>
-      <c r="K43">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="44" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B44" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*200</v>
-      </c>
-      <c r="F44" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-200V</v>
-      </c>
-      <c r="K44">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="45" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B45" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*236</v>
-      </c>
-      <c r="F45" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-236V</v>
-      </c>
-      <c r="K45">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="46" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B46" t="str">
-        <f t="shared" si="0"/>
-        <v>g[_]*600</v>
-      </c>
-      <c r="F46" t="str">
-        <f t="shared" si="1"/>
-        <v>Grid-600V</v>
-      </c>
-      <c r="K46">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="47" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B47" t="s">
-        <v>90</v>
-      </c>
-      <c r="F47" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="48" spans="2:11" x14ac:dyDescent="0.45">
-      <c r="B48" t="s">
-        <v>79</v>
-      </c>
-      <c r="F48" t="s">
-        <v>80</v>
       </c>
     </row>
   </sheetData>

</xml_diff>